<commit_message>
Minor improvement to GetClauseVar and fixed a bug in IncrementalSolve.
</commit_message>
<xml_diff>
--- a/Timings.xlsx
+++ b/Timings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A2188B4-A12C-4FCC-8529-A51B13CCCAB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27E9F2C-BFC6-4EB2-8954-8766A6001E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-150" yWindow="885" windowWidth="28950" windowHeight="14595" xr2:uid="{8E1E5196-6F02-42B2-AA15-40F94B4B1E52}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>HasFP</t>
   </si>
@@ -72,6 +72,33 @@
   </si>
   <si>
     <t>Psi3b</t>
+  </si>
+  <si>
+    <t>Solver</t>
+  </si>
+  <si>
+    <t>minisat</t>
+  </si>
+  <si>
+    <t>minisatKiel</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>shuffled</t>
+  </si>
+  <si>
+    <t>sorted</t>
+  </si>
+  <si>
+    <t>original</t>
+  </si>
+  <si>
+    <t>reversed</t>
+  </si>
+  <si>
+    <t>window</t>
   </si>
 </sst>
 </file>
@@ -206,7 +233,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$13:$A$32</c:f>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -275,7 +302,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$13:$B$32</c:f>
+              <c:f>Sheet1!$B$14:$B$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -366,7 +393,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$13:$A$32</c:f>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -435,7 +462,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$13:$C$32</c:f>
+              <c:f>Sheet1!$C$14:$C$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -526,7 +553,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$13:$A$32</c:f>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -595,7 +622,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$13:$D$32</c:f>
+              <c:f>Sheet1!$D$14:$D$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -686,7 +713,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$13:$A$32</c:f>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -755,7 +782,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$E$13:$E$32</c:f>
+              <c:f>Sheet1!$E$14:$E$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -846,7 +873,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$13:$A$32</c:f>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -915,7 +942,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$F$13:$F$32</c:f>
+              <c:f>Sheet1!$F$14:$F$33</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -986,6 +1013,814 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-0E96-420C-AC3A-B72C4E9BDF3A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$G$14:$G$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-4.8562196370224804</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.3925863805310801</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4.0798550702707601</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3.6245599654151199</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-3.3895915941056201</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-3.0440338976940802</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-2.8329400461815899</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-2.2488864176712302</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2.1306501698143001</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-1.7986161267831999</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-1.8023065320488401</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-1.41721556226005</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.90043264032657999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.89023915964816602</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-0.40624084817060002</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.1431978566558793E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.92172951587886098</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.37491612677564801</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.89714000954294804</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.58693514303776495</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3CEE-49B5-BEC2-895D09A14562}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$H$14:$H$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-5.0209553508828799</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.4399411374737197</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4.1596563944739797</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3.5074061874802802</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-3.5318219325958702</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-3.4469381133174699</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-3.25966198586611</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-2.0595784059768798</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2.9159717352290202</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-2.6920996689467702</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-2.4169328618379202</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-1.83789044495408</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-2.34536507212465</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.79407686161559299</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-1.8996090198933999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.41385243646303</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-1.23074675343647</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.103406673343288</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.4071046132271501</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-0.22687775332399701</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-3CEE-49B5-BEC2-895D09A14562}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$14:$I$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-5.4144921728534703</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-5.0015665997501602</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4.7915379925094204</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-4.4775155467899399</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.3328492586653802</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.1375279373887404</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-3.90935314161643</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-3.7724924855417798</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-3.6720507794262498</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3.56345810856492</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-3.5782566112986101</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-3.4520379509805101</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-3.2914911260832</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-3.1606525339371601</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-3.0463034024624198</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-2.99838101181061</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-2.8761271933569899</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-2.7560488093320599</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-2.68614219935459</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-2.2785754165298799</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-3CEE-49B5-BEC2-895D09A14562}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$J$14:$J$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-4.7733831432751597</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.4000600656150599</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4.0336489179212203</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3.7179384645844999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-3.5492514370389898</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-2.9648389238209498</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-2.7408501863755999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-2.4189309558511298</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2.0284621516011798</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-1.8729930342157901</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-2.78763705302064</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-2.2194502012477302</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-2.4403724952721002</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-1.96102297877057</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-2.02027449190496</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-2.2983997472170099</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-2.1190091266387499</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-1.8142869223751701</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.40304036636715</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-2.11570457055217</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-3CEE-49B5-BEC2-895D09A14562}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="9"/>
+          <c:order val="9"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$14:$A$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$14:$K$33</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-5.4385506902088299</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-5.3076774800466904</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-5.0927749472074701</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-4.7419105193523396</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.6145855006319998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.44007712952516</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-4.3341197238154203</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-4.3635137431465099</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-4.27265276363394</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-4.0901921186220296</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-3.99127942902245</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-3.8777100316628599</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-3.7329735508987199</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-3.5886712019549498</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-3.5084665768220802</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-3.4712256093798599</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-3.3107791930331998</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-3.13797833280936</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-3.24063807024852</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-3.1335356074289198</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-3CEE-49B5-BEC2-895D09A14562}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1132,37 +1967,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1767,16 +2571,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>404811</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>128586</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>442911</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>42861</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>200024</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>133349</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>238124</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>47624</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2121,517 +2925,942 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14293D77-34DA-4666-B69A-8EC274C7BBDD}">
-  <dimension ref="A2:F32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>1</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="1"/>
+      <c r="D8" s="2"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14">
         <v>0.01</v>
       </c>
-      <c r="B13">
+      <c r="B14">
         <v>-4.8307368539008015</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>-4.7689037557560026</v>
       </c>
-      <c r="D13">
+      <c r="D14">
         <v>-4.7694832643159897</v>
       </c>
-      <c r="E13">
+      <c r="E14">
         <v>-4.5838031146277496</v>
       </c>
-      <c r="F13">
+      <c r="F14">
         <v>-4.6859454669984704</v>
       </c>
+      <c r="G14">
+        <v>-4.8562196370224804</v>
+      </c>
+      <c r="H14">
+        <v>-5.0209553508828799</v>
+      </c>
+      <c r="I14">
+        <v>-5.4144921728534703</v>
+      </c>
+      <c r="J14">
+        <v>-4.7733831432751597</v>
+      </c>
+      <c r="K14">
+        <v>-5.4385506902088299</v>
+      </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15">
         <v>0.02</v>
       </c>
-      <c r="B14">
+      <c r="B15">
         <v>-4.4255924032366796</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>-4.3036835200256718</v>
       </c>
-      <c r="D14">
+      <c r="D15">
         <v>-4.3025744650196902</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <v>-4.1121972309262897</v>
       </c>
-      <c r="F14">
+      <c r="F15">
         <v>-4.1510399135668798</v>
       </c>
+      <c r="G15">
+        <v>-4.3925863805310801</v>
+      </c>
+      <c r="H15">
+        <v>-4.4399411374737197</v>
+      </c>
+      <c r="I15">
+        <v>-5.0015665997501602</v>
+      </c>
+      <c r="J15">
+        <v>-4.4000600656150599</v>
+      </c>
+      <c r="K15">
+        <v>-5.3076774800466904</v>
+      </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16">
         <v>0.03</v>
       </c>
-      <c r="B15">
+      <c r="B16">
         <v>-4.110251688065734</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>-3.9832867639963889</v>
       </c>
-      <c r="D15">
+      <c r="D16">
         <v>-3.6911619396000002</v>
       </c>
-      <c r="E15">
+      <c r="E16">
         <v>-3.53935263299564</v>
       </c>
-      <c r="F15">
+      <c r="F16">
         <v>-3.7323784177521402</v>
       </c>
+      <c r="G16">
+        <v>-4.0798550702707601</v>
+      </c>
+      <c r="H16">
+        <v>-4.1596563944739797</v>
+      </c>
+      <c r="I16">
+        <v>-4.7915379925094204</v>
+      </c>
+      <c r="J16">
+        <v>-4.0336489179212203</v>
+      </c>
+      <c r="K16">
+        <v>-5.0927749472074701</v>
+      </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>0.04</v>
       </c>
-      <c r="B16">
+      <c r="B17">
         <v>-3.6970521545202044</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>-3.6199584789622468</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <v>-3.4532406815379102</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <v>-3.1360652777840898</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <v>-3.4366077110931101</v>
       </c>
+      <c r="G17">
+        <v>-3.6245599654151199</v>
+      </c>
+      <c r="H17">
+        <v>-3.5074061874802802</v>
+      </c>
+      <c r="I17">
+        <v>-4.4775155467899399</v>
+      </c>
+      <c r="J17">
+        <v>-3.7179384645844999</v>
+      </c>
+      <c r="K17">
+        <v>-4.7419105193523396</v>
+      </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18">
         <v>0.05</v>
       </c>
-      <c r="B17">
+      <c r="B18">
         <v>-3.4621822371078972</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>-3.3005144255949244</v>
       </c>
-      <c r="D17">
+      <c r="D18">
         <v>-3.2043888732610002</v>
       </c>
-      <c r="E17">
+      <c r="E18">
         <v>-2.6039318327494101</v>
       </c>
-      <c r="F17">
+      <c r="F18">
         <v>-3.1905734768463101</v>
       </c>
+      <c r="G18">
+        <v>-3.3895915941056201</v>
+      </c>
+      <c r="H18">
+        <v>-3.5318219325958702</v>
+      </c>
+      <c r="I18">
+        <v>-4.3328492586653802</v>
+      </c>
+      <c r="J18">
+        <v>-3.5492514370389898</v>
+      </c>
+      <c r="K18">
+        <v>-4.6145855006319998</v>
+      </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19">
         <v>0.06</v>
       </c>
-      <c r="B18">
+      <c r="B19">
         <v>-2.8796272114971746</v>
       </c>
-      <c r="C18">
+      <c r="C19">
         <v>-3.0293230801045641</v>
       </c>
-      <c r="D18">
+      <c r="D19">
         <v>-2.9025872333979601</v>
       </c>
-      <c r="E18">
+      <c r="E19">
         <v>-1.8719042753614299</v>
       </c>
-      <c r="F18">
+      <c r="F19">
         <v>-2.6579670367129098</v>
       </c>
+      <c r="G19">
+        <v>-3.0440338976940802</v>
+      </c>
+      <c r="H19">
+        <v>-3.4469381133174699</v>
+      </c>
+      <c r="I19">
+        <v>-4.1375279373887404</v>
+      </c>
+      <c r="J19">
+        <v>-2.9648389238209498</v>
+      </c>
+      <c r="K19">
+        <v>-4.44007712952516</v>
+      </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="B19">
+      <c r="B20">
         <v>-2.9128863722275238</v>
       </c>
-      <c r="C19">
+      <c r="C20">
         <v>-2.6087319365318491</v>
       </c>
-      <c r="D19">
+      <c r="D20">
         <v>-2.5309623778511199</v>
       </c>
-      <c r="E19">
+      <c r="E20">
         <v>-1.8384349707952701</v>
       </c>
-      <c r="F19">
+      <c r="F20">
         <v>-2.5814763090176802</v>
       </c>
+      <c r="G20">
+        <v>-2.8329400461815899</v>
+      </c>
+      <c r="H20">
+        <v>-3.25966198586611</v>
+      </c>
+      <c r="I20">
+        <v>-3.90935314161643</v>
+      </c>
+      <c r="J20">
+        <v>-2.7408501863755999</v>
+      </c>
+      <c r="K20">
+        <v>-4.3341197238154203</v>
+      </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21">
         <v>0.08</v>
       </c>
-      <c r="B20">
+      <c r="B21">
         <v>-2.514490681135654</v>
       </c>
-      <c r="C20">
+      <c r="C21">
         <v>-2.5475536293810466</v>
       </c>
-      <c r="D20">
+      <c r="D21">
         <v>-2.5562423990081</v>
       </c>
-      <c r="E20">
+      <c r="E21">
         <v>-1.2631876523399801</v>
       </c>
-      <c r="F20">
+      <c r="F21">
         <v>-2.3670387049769199</v>
       </c>
+      <c r="G21">
+        <v>-2.2488864176712302</v>
+      </c>
+      <c r="H21">
+        <v>-2.0595784059768798</v>
+      </c>
+      <c r="I21">
+        <v>-3.7724924855417798</v>
+      </c>
+      <c r="J21">
+        <v>-2.4189309558511298</v>
+      </c>
+      <c r="K21">
+        <v>-4.3635137431465099</v>
+      </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22">
         <v>0.09</v>
       </c>
-      <c r="B21">
+      <c r="B22">
         <v>-1.9915534241236252</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>-2.5387073413127021</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>-2.1480963254633099</v>
       </c>
-      <c r="E21">
+      <c r="E22">
         <v>-1.3670330971167901</v>
       </c>
-      <c r="F21">
+      <c r="F22">
         <v>-2.0385593673956701</v>
       </c>
+      <c r="G22">
+        <v>-2.1306501698143001</v>
+      </c>
+      <c r="H22">
+        <v>-2.9159717352290202</v>
+      </c>
+      <c r="I22">
+        <v>-3.6720507794262498</v>
+      </c>
+      <c r="J22">
+        <v>-2.0284621516011798</v>
+      </c>
+      <c r="K22">
+        <v>-4.27265276363394</v>
+      </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23">
         <v>0.1</v>
       </c>
-      <c r="B22">
+      <c r="B23">
         <v>-1.7791419360065197</v>
       </c>
-      <c r="C22">
+      <c r="C23">
         <v>-1.9736773772250085</v>
       </c>
-      <c r="D22">
+      <c r="D23">
         <v>-1.73906901751452</v>
       </c>
-      <c r="E22">
+      <c r="E23">
         <v>-1.0344995303405999</v>
       </c>
-      <c r="F22">
+      <c r="F23">
         <v>-1.8106409895966999</v>
       </c>
+      <c r="G23">
+        <v>-1.7986161267831999</v>
+      </c>
+      <c r="H23">
+        <v>-2.6920996689467702</v>
+      </c>
+      <c r="I23">
+        <v>-3.56345810856492</v>
+      </c>
+      <c r="J23">
+        <v>-1.8729930342157901</v>
+      </c>
+      <c r="K23">
+        <v>-4.0901921186220296</v>
+      </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24">
         <v>0.11</v>
       </c>
-      <c r="B23">
+      <c r="B24">
         <v>-1.4536593639422248</v>
       </c>
-      <c r="C23">
+      <c r="C24">
         <v>-1.5679876215853752</v>
       </c>
-      <c r="D23">
+      <c r="D24">
         <v>-1.6641613698450499</v>
       </c>
-      <c r="E23">
+      <c r="E24">
         <v>-0.76487758847231602</v>
       </c>
-      <c r="F23">
+      <c r="F24">
         <v>-0.975796148686217</v>
       </c>
+      <c r="G24">
+        <v>-1.8023065320488401</v>
+      </c>
+      <c r="H24">
+        <v>-2.4169328618379202</v>
+      </c>
+      <c r="I24">
+        <v>-3.5782566112986101</v>
+      </c>
+      <c r="J24">
+        <v>-2.78763705302064</v>
+      </c>
+      <c r="K24">
+        <v>-3.99127942902245</v>
+      </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25">
         <v>0.12</v>
       </c>
-      <c r="B24">
+      <c r="B25">
         <v>-1.0854957558921552</v>
       </c>
-      <c r="C24">
+      <c r="C25">
         <v>-0.94862907090861848</v>
       </c>
-      <c r="D24">
+      <c r="D25">
         <v>-1.2631858075422999</v>
       </c>
-      <c r="E24">
+      <c r="E25">
         <v>-0.39274166143660799</v>
       </c>
-      <c r="F24">
+      <c r="F25">
         <v>-0.41471224592896999</v>
       </c>
+      <c r="G25">
+        <v>-1.41721556226005</v>
+      </c>
+      <c r="H25">
+        <v>-1.83789044495408</v>
+      </c>
+      <c r="I25">
+        <v>-3.4520379509805101</v>
+      </c>
+      <c r="J25">
+        <v>-2.2194502012477302</v>
+      </c>
+      <c r="K25">
+        <v>-3.8777100316628599</v>
+      </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26">
         <v>0.13</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <v>-0.70414129079952792</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>-1.0009984982444087</v>
       </c>
-      <c r="D25">
+      <c r="D26">
         <v>-0.83929119029126997</v>
       </c>
-      <c r="E25">
+      <c r="E26">
         <v>-0.16041130211419599</v>
       </c>
-      <c r="F25">
+      <c r="F26">
         <v>-0.47647930902596802</v>
       </c>
+      <c r="G26">
+        <v>-0.90043264032657999</v>
+      </c>
+      <c r="H26">
+        <v>-2.34536507212465</v>
+      </c>
+      <c r="I26">
+        <v>-3.2914911260832</v>
+      </c>
+      <c r="J26">
+        <v>-2.4403724952721002</v>
+      </c>
+      <c r="K26">
+        <v>-3.7329735508987199</v>
+      </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27">
         <v>0.14000000000000001</v>
       </c>
-      <c r="B26">
+      <c r="B27">
         <v>-0.62047702037881869</v>
       </c>
-      <c r="C26">
+      <c r="C27">
         <v>-0.5104019200204698</v>
       </c>
-      <c r="D26">
+      <c r="D27">
         <v>-0.949949441896493</v>
       </c>
-      <c r="E26">
+      <c r="E27">
         <v>8.79322777668686E-2</v>
       </c>
-      <c r="F26">
+      <c r="F27">
         <v>-0.101210295332381</v>
       </c>
+      <c r="G27">
+        <v>-0.89023915964816602</v>
+      </c>
+      <c r="H27">
+        <v>-0.79407686161559299</v>
+      </c>
+      <c r="I27">
+        <v>-3.1606525339371601</v>
+      </c>
+      <c r="J27">
+        <v>-1.96102297877057</v>
+      </c>
+      <c r="K27">
+        <v>-3.5886712019549498</v>
+      </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28">
         <v>0.15</v>
       </c>
-      <c r="B27">
+      <c r="B28">
         <v>-0.47647062397143453</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>-0.66055306448410078</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <v>-0.352813633263108</v>
       </c>
-      <c r="E27">
+      <c r="E28">
         <v>0.194961607946224</v>
       </c>
-      <c r="F27">
+      <c r="F28">
         <v>0.50147617423798996</v>
       </c>
+      <c r="G28">
+        <v>-0.40624084817060002</v>
+      </c>
+      <c r="H28">
+        <v>-1.8996090198933999</v>
+      </c>
+      <c r="I28">
+        <v>-3.0463034024624198</v>
+      </c>
+      <c r="J28">
+        <v>-2.02027449190496</v>
+      </c>
+      <c r="K28">
+        <v>-3.5084665768220802</v>
+      </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29">
         <v>0.16</v>
       </c>
-      <c r="B28">
+      <c r="B29">
         <v>0.27177532719159753</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>0.13717880255052764</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>-5.26656487444861E-2</v>
       </c>
-      <c r="E28">
+      <c r="E29">
         <v>1.01437554756363</v>
       </c>
-      <c r="F28">
+      <c r="F29">
         <v>0.86238216378425003</v>
       </c>
+      <c r="G29">
+        <v>7.1431978566558793E-2</v>
+      </c>
+      <c r="H29">
+        <v>-1.41385243646303</v>
+      </c>
+      <c r="I29">
+        <v>-2.99838101181061</v>
+      </c>
+      <c r="J29">
+        <v>-2.2983997472170099</v>
+      </c>
+      <c r="K29">
+        <v>-3.4712256093798599</v>
+      </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30">
         <v>0.17</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <v>0.76455816866535642</v>
       </c>
-      <c r="C29">
+      <c r="C30">
         <v>0.32993190194160488</v>
       </c>
-      <c r="D29">
+      <c r="D30">
         <v>0.29868867032747698</v>
       </c>
-      <c r="E29">
+      <c r="E30">
         <v>1.2761607122462499</v>
       </c>
-      <c r="F29">
+      <c r="F30">
         <v>0.54897646959278101</v>
       </c>
+      <c r="G30">
+        <v>0.92172951587886098</v>
+      </c>
+      <c r="H30">
+        <v>-1.23074675343647</v>
+      </c>
+      <c r="I30">
+        <v>-2.8761271933569899</v>
+      </c>
+      <c r="J30">
+        <v>-2.1190091266387499</v>
+      </c>
+      <c r="K30">
+        <v>-3.3107791930331998</v>
+      </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31">
         <v>0.18</v>
       </c>
-      <c r="B30">
+      <c r="B31">
         <v>0.33706564977038972</v>
       </c>
-      <c r="C30">
+      <c r="C31">
         <v>0.52805979942377623</v>
       </c>
-      <c r="D30">
+      <c r="D31">
         <v>0.23765414494185499</v>
       </c>
-      <c r="E30">
+      <c r="E31">
         <v>1.6393955311711199</v>
       </c>
-      <c r="F30">
+      <c r="F31">
         <v>1.5518147374342</v>
       </c>
+      <c r="G31">
+        <v>0.37491612677564801</v>
+      </c>
+      <c r="H31">
+        <v>0.103406673343288</v>
+      </c>
+      <c r="I31">
+        <v>-2.7560488093320599</v>
+      </c>
+      <c r="J31">
+        <v>-1.8142869223751701</v>
+      </c>
+      <c r="K31">
+        <v>-3.13797833280936</v>
+      </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32">
         <v>0.19</v>
       </c>
-      <c r="B31">
+      <c r="B32">
         <v>0.4764380897320778</v>
       </c>
-      <c r="C31">
+      <c r="C32">
         <v>0.67367926517295518</v>
       </c>
-      <c r="D31">
+      <c r="D32">
         <v>1.08596574784003</v>
       </c>
-      <c r="E31">
+      <c r="E32">
         <v>1.8672370024028699</v>
       </c>
-      <c r="F31">
+      <c r="F32">
         <v>1.6669005313852401</v>
       </c>
+      <c r="G32">
+        <v>0.89714000954294804</v>
+      </c>
+      <c r="H32">
+        <v>1.4071046132271501</v>
+      </c>
+      <c r="I32">
+        <v>-2.68614219935459</v>
+      </c>
+      <c r="J32">
+        <v>-1.40304036636715</v>
+      </c>
+      <c r="K32">
+        <v>-3.24063807024852</v>
+      </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33">
         <v>0.2</v>
       </c>
-      <c r="B32">
+      <c r="B33">
         <v>0.85130254659390681</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>0.74885374900326585</v>
       </c>
-      <c r="D32">
+      <c r="D33">
         <v>0.25866053252760202</v>
       </c>
-      <c r="E32">
+      <c r="E33">
         <v>1.24022881503895</v>
       </c>
-      <c r="F32">
+      <c r="F33">
         <v>1.88066715213785</v>
+      </c>
+      <c r="G33">
+        <v>0.58693514303776495</v>
+      </c>
+      <c r="H33">
+        <v>-0.22687775332399701</v>
+      </c>
+      <c r="I33">
+        <v>-2.2785754165298799</v>
+      </c>
+      <c r="J33">
+        <v>-2.11570457055217</v>
+      </c>
+      <c r="K33">
+        <v>-3.1335356074289198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>